<commit_message>
Actualizar precios de impovar.xlsx (alza +5.45%)
Mismos 25 códigos y descripciones, mismo formato de planilla trimestral;
solo se actualizan los precios por tira/metro con la nueva cotización.
</commit_message>
<xml_diff>
--- a/impovar.xlsx
+++ b/impovar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://abastible-my.sharepoint.com/personal/daniel_villalobos_abastible_cl/Documents/ABASTIBLE/PROYECTOS DANIEL/NOTA DE VENTA/NOTA-VENTA-V5/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_CB51073D694B4E468518322F25FC54239F81EABE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96F57087-F41F-4775-AFC0-5A7FD269136C}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_CB51073D694B4E468518322F25FC54239F81EABE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C99CF37-38B0-4831-B6F3-39CB4D271943}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MATERIAL CAÑERIAS" sheetId="4" r:id="rId1"/>
@@ -158,11 +158,39 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -171,15 +199,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda [0]" xfId="1" builtinId="7"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="9">
     <dxf>
       <font>
         <b val="0"/>
@@ -197,6 +227,11 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -215,6 +250,91 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="0"/>
+        </left>
+        <right style="thin">
+          <color theme="0"/>
+        </right>
+        <top style="thin">
+          <color theme="0"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -230,18 +350,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9A9BC17C-D6CF-49C5-8D0F-755D7EB56C1D}" name="Tabla1" displayName="Tabla1" ref="D6:J31" totalsRowShown="0">
-  <autoFilter ref="D6:J31" xr:uid="{9A9BC17C-D6CF-49C5-8D0F-755D7EB56C1D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{68B94CD0-D4A9-4C0B-ADAC-ABF8C1279EE4}" name="Tabla1" displayName="Tabla1" ref="D6:J31" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="D6:J31" xr:uid="{68B94CD0-D4A9-4C0B-ADAC-ABF8C1279EE4}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{BB337050-0FCF-4268-8FA5-C2F121668045}" name="DESCRIPCIÓN"/>
-    <tableColumn id="2" xr3:uid="{58CAB42F-E925-47B7-B2BA-0D0216D3066E}" name="CODIGO"/>
-    <tableColumn id="7" xr3:uid="{1179C10A-41BF-449E-AA96-9BD707046D57}" name="CATEGORIA"/>
-    <tableColumn id="3" xr3:uid="{F8616042-8AFA-46E4-B850-F04B8F575DCF}" name="MONEDA"/>
-    <tableColumn id="4" xr3:uid="{CB56C481-711F-4129-B95A-9FD6AB3EF51B}" name="TIRA o ROLLO [Mt.]"/>
-    <tableColumn id="5" xr3:uid="{589ED3D9-0B69-4014-8DDB-842D3B0AF9E2}" name="PRECIO POR TIRA [CLP/(tira o rollo)]" dataDxfId="1" dataCellStyle="Moneda [0]"/>
-    <tableColumn id="6" xr3:uid="{CA57DB04-C495-419D-A705-AD75636E4B10}" name="PRECIO POR METRO [CLP/Mt.]" dataDxfId="0" dataCellStyle="Moneda [0]"/>
+    <tableColumn id="1" xr3:uid="{297555F9-46F3-4D4A-ACAE-12F3FE0D0D88}" name="DESCRIPCIÓN" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{CD6EEAF1-B02C-4A94-B003-CE532EFF6B09}" name="CODIGO" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{88C8A75D-6508-4A3B-AA43-B4ED5445E5DF}" name="CATEGORIA" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{F57C2549-C9E0-4234-A091-C30A9DC95E40}" name="MONEDA" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{F3C8260F-F02E-40AF-A198-AEDEC1FDCF92}" name="TIRA o ROLLO [Mt.]" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{7E658286-9D47-484B-A8BE-1855DC378DD7}" name="PRECIO POR TIRA [CLP/(tira o rollo)]" dataDxfId="1" dataCellStyle="Moneda [0]"/>
+    <tableColumn id="7" xr3:uid="{277BC4FC-E057-4CFA-AB6A-DB93BC93B269}" name="PRECIO POR METRO [CLP/Mt.]" dataDxfId="0" dataCellStyle="Moneda [0]"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -530,7 +650,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B27436D4-AFED-4A83-B6AF-2AA972709B69}">
-  <dimension ref="D6:J31"/>
+  <dimension ref="C6:J31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="37.7109375" bestFit="1" customWidth="1"/>
@@ -542,7 +662,7 @@
     <col min="10" max="10" width="29.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="6" spans="4:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:10" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
         <v>25</v>
       </c>
@@ -565,14 +685,17 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="4:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C7">
+        <v>1</v>
+      </c>
       <c r="D7" t="s">
         <v>8</v>
       </c>
       <c r="E7">
         <v>24812</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G7" t="s">
@@ -581,21 +704,24 @@
       <c r="H7">
         <v>6</v>
       </c>
-      <c r="I7" s="1">
-        <v>23887.875</v>
-      </c>
-      <c r="J7" s="1">
-        <v>3981.3125</v>
-      </c>
-    </row>
-    <row r="8" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I7" s="2">
+        <v>25190.85</v>
+      </c>
+      <c r="J7" s="2">
+        <v>4198.4749999999995</v>
+      </c>
+    </row>
+    <row r="8" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C8">
+        <v>2</v>
+      </c>
       <c r="D8" t="s">
         <v>9</v>
       </c>
       <c r="E8">
         <v>24807</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G8" t="s">
@@ -604,21 +730,24 @@
       <c r="H8">
         <v>6</v>
       </c>
-      <c r="I8" s="1">
-        <v>34127.5</v>
-      </c>
-      <c r="J8" s="1">
-        <v>5687.916666666667</v>
-      </c>
-    </row>
-    <row r="9" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I8" s="2">
+        <v>35989</v>
+      </c>
+      <c r="J8" s="2">
+        <v>5998.166666666667</v>
+      </c>
+    </row>
+    <row r="9" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C9">
+        <v>3</v>
+      </c>
       <c r="D9" t="s">
         <v>10</v>
       </c>
       <c r="E9">
         <v>24811</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G9" t="s">
@@ -627,21 +756,24 @@
       <c r="H9">
         <v>6</v>
       </c>
-      <c r="I9" s="1">
-        <v>54309.75</v>
-      </c>
-      <c r="J9" s="1">
-        <v>9051.625</v>
-      </c>
-    </row>
-    <row r="10" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I9" s="2">
+        <v>57272.1</v>
+      </c>
+      <c r="J9" s="2">
+        <v>9545.35</v>
+      </c>
+    </row>
+    <row r="10" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C10">
+        <v>4</v>
+      </c>
       <c r="D10" t="s">
         <v>11</v>
       </c>
       <c r="E10">
         <v>24806</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G10" t="s">
@@ -650,21 +782,24 @@
       <c r="H10">
         <v>6</v>
       </c>
-      <c r="I10" s="1">
-        <v>78647.25</v>
-      </c>
-      <c r="J10" s="1">
-        <v>13107.875</v>
-      </c>
-    </row>
-    <row r="11" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I10" s="2">
+        <v>82937.099999999991</v>
+      </c>
+      <c r="J10" s="2">
+        <v>13822.849999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C11">
+        <v>5</v>
+      </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11">
         <v>24805</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G11" t="s">
@@ -673,21 +808,24 @@
       <c r="H11">
         <v>6</v>
       </c>
-      <c r="I11" s="1">
-        <v>106532.25</v>
-      </c>
-      <c r="J11" s="1">
-        <v>17755.375</v>
-      </c>
-    </row>
-    <row r="12" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I11" s="2">
+        <v>112343.09999999999</v>
+      </c>
+      <c r="J11" s="2">
+        <v>18723.849999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C12">
+        <v>6</v>
+      </c>
       <c r="D12" t="s">
         <v>13</v>
       </c>
       <c r="E12">
         <v>24804</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G12" t="s">
@@ -696,21 +834,24 @@
       <c r="H12">
         <v>6</v>
       </c>
-      <c r="I12" s="1">
-        <v>139317.75</v>
-      </c>
-      <c r="J12" s="1">
-        <v>23219.625</v>
-      </c>
-    </row>
-    <row r="13" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I12" s="2">
+        <v>146916.9</v>
+      </c>
+      <c r="J12" s="2">
+        <v>24486.149999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C13">
+        <v>7</v>
+      </c>
       <c r="D13" t="s">
         <v>14</v>
       </c>
       <c r="E13">
         <v>24809</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G13" t="s">
@@ -719,21 +860,24 @@
       <c r="H13">
         <v>6</v>
       </c>
-      <c r="I13" s="1">
-        <v>214201.625</v>
-      </c>
-      <c r="J13" s="1">
-        <v>35700.270833333336</v>
-      </c>
-    </row>
-    <row r="14" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I13" s="2">
+        <v>225885.35</v>
+      </c>
+      <c r="J13" s="2">
+        <v>37647.558333333334</v>
+      </c>
+    </row>
+    <row r="14" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C14">
+        <v>8</v>
+      </c>
       <c r="D14" t="s">
         <v>15</v>
       </c>
       <c r="E14">
         <v>24808</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G14" t="s">
@@ -742,21 +886,24 @@
       <c r="H14">
         <v>6</v>
       </c>
-      <c r="I14" s="1">
-        <v>317739.125</v>
-      </c>
-      <c r="J14" s="1">
-        <v>52956.520833333336</v>
-      </c>
-    </row>
-    <row r="15" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I14" s="2">
+        <v>335070.34999999998</v>
+      </c>
+      <c r="J14" s="2">
+        <v>55845.058333333327</v>
+      </c>
+    </row>
+    <row r="15" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C15">
+        <v>9</v>
+      </c>
       <c r="D15" t="s">
         <v>16</v>
       </c>
       <c r="E15">
         <v>24810</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G15" t="s">
@@ -765,21 +912,24 @@
       <c r="H15">
         <v>6</v>
       </c>
-      <c r="I15" s="1">
-        <v>425475.875</v>
-      </c>
-      <c r="J15" s="1">
-        <v>70912.645833333328</v>
-      </c>
-    </row>
-    <row r="16" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I15" s="2">
+        <v>448683.64999999997</v>
+      </c>
+      <c r="J15" s="2">
+        <v>74780.608333333323</v>
+      </c>
+    </row>
+    <row r="16" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C16">
+        <v>10</v>
+      </c>
       <c r="D16" t="s">
         <v>17</v>
       </c>
       <c r="E16">
         <v>24822</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G16" t="s">
@@ -788,21 +938,24 @@
       <c r="H16">
         <v>6</v>
       </c>
-      <c r="I16" s="1">
-        <v>694743.5</v>
-      </c>
-      <c r="J16" s="1">
-        <v>115790.58333333333</v>
-      </c>
-    </row>
-    <row r="17" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I16" s="2">
+        <v>732638.6</v>
+      </c>
+      <c r="J16" s="2">
+        <v>122106.43333333333</v>
+      </c>
+    </row>
+    <row r="17" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C17">
+        <v>11</v>
+      </c>
       <c r="D17" t="s">
         <v>18</v>
       </c>
       <c r="E17">
         <v>24974</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G17" t="s">
@@ -811,21 +964,24 @@
       <c r="H17">
         <v>18</v>
       </c>
-      <c r="I17" s="1">
-        <v>74244.5</v>
-      </c>
-      <c r="J17" s="1">
-        <v>4124.6944444444443</v>
-      </c>
-    </row>
-    <row r="18" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I17" s="2">
+        <v>78294.2</v>
+      </c>
+      <c r="J17" s="2">
+        <v>4349.6777777777779</v>
+      </c>
+    </row>
+    <row r="18" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C18">
+        <v>12</v>
+      </c>
       <c r="D18" t="s">
         <v>19</v>
       </c>
       <c r="E18">
         <v>24975</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G18" t="s">
@@ -834,21 +990,24 @@
       <c r="H18">
         <v>18</v>
       </c>
-      <c r="I18" s="1">
-        <v>106565.25</v>
-      </c>
-      <c r="J18" s="1">
-        <v>5920.291666666667</v>
-      </c>
-    </row>
-    <row r="19" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I18" s="2">
+        <v>112377.9</v>
+      </c>
+      <c r="J18" s="2">
+        <v>6243.2166666666662</v>
+      </c>
+    </row>
+    <row r="19" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C19">
+        <v>13</v>
+      </c>
       <c r="D19" t="s">
         <v>20</v>
       </c>
       <c r="E19">
         <v>24973</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G19" t="s">
@@ -857,21 +1016,24 @@
       <c r="H19">
         <v>18</v>
       </c>
-      <c r="I19" s="1">
-        <v>168768.875</v>
-      </c>
-      <c r="J19" s="1">
-        <v>9376.0486111111113</v>
-      </c>
-    </row>
-    <row r="20" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I19" s="2">
+        <v>177974.44999999998</v>
+      </c>
+      <c r="J19" s="2">
+        <v>9887.4694444444431</v>
+      </c>
+    </row>
+    <row r="20" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C20">
+        <v>14</v>
+      </c>
       <c r="D20" t="s">
         <v>21</v>
       </c>
       <c r="E20">
         <v>24978</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G20" t="s">
@@ -880,21 +1042,24 @@
       <c r="H20">
         <v>6</v>
       </c>
-      <c r="I20" s="1">
-        <v>27198.875</v>
-      </c>
-      <c r="J20" s="1">
-        <v>4533.145833333333</v>
-      </c>
-    </row>
-    <row r="21" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I20" s="2">
+        <v>28682.45</v>
+      </c>
+      <c r="J20" s="2">
+        <v>4780.4083333333338</v>
+      </c>
+    </row>
+    <row r="21" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C21">
+        <v>15</v>
+      </c>
       <c r="D21" t="s">
         <v>22</v>
       </c>
       <c r="E21">
         <v>24992</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G21" t="s">
@@ -903,21 +1068,24 @@
       <c r="H21">
         <v>6</v>
       </c>
-      <c r="I21" s="1">
-        <v>39304.375</v>
-      </c>
-      <c r="J21" s="1">
-        <v>6550.729166666667</v>
-      </c>
-    </row>
-    <row r="22" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I21" s="2">
+        <v>41448.25</v>
+      </c>
+      <c r="J21" s="2">
+        <v>6908.041666666667</v>
+      </c>
+    </row>
+    <row r="22" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C22">
+        <v>16</v>
+      </c>
       <c r="D22" t="s">
         <v>23</v>
       </c>
       <c r="E22">
         <v>24977</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G22" t="s">
@@ -926,21 +1094,24 @@
       <c r="H22">
         <v>6</v>
       </c>
-      <c r="I22" s="1">
-        <v>60541.25</v>
-      </c>
-      <c r="J22" s="1">
-        <v>10090.208333333334</v>
-      </c>
-    </row>
-    <row r="23" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I22" s="2">
+        <v>63843.5</v>
+      </c>
+      <c r="J22" s="2">
+        <v>10640.583333333334</v>
+      </c>
+    </row>
+    <row r="23" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C23">
+        <v>17</v>
+      </c>
       <c r="D23" t="s">
         <v>24</v>
       </c>
       <c r="E23">
         <v>24993</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G23" t="s">
@@ -949,21 +1120,24 @@
       <c r="H23">
         <v>6</v>
       </c>
-      <c r="I23" s="1">
-        <v>86026.875</v>
-      </c>
-      <c r="J23" s="1">
-        <v>14337.8125</v>
-      </c>
-    </row>
-    <row r="24" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I23" s="2">
+        <v>90719.25</v>
+      </c>
+      <c r="J23" s="2">
+        <v>15119.875</v>
+      </c>
+    </row>
+    <row r="24" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C24">
+        <v>18</v>
+      </c>
       <c r="D24" t="s">
         <v>0</v>
       </c>
       <c r="E24">
         <v>24803</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G24" t="s">
@@ -972,21 +1146,24 @@
       <c r="H24">
         <v>6</v>
       </c>
-      <c r="I24" s="1">
-        <v>34966.25</v>
-      </c>
-      <c r="J24" s="1">
-        <v>5827.708333333333</v>
-      </c>
-    </row>
-    <row r="25" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I24" s="2">
+        <v>36873.5</v>
+      </c>
+      <c r="J24" s="2">
+        <v>6145.583333333333</v>
+      </c>
+    </row>
+    <row r="25" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C25">
+        <v>19</v>
+      </c>
       <c r="D25" t="s">
         <v>1</v>
       </c>
       <c r="E25">
         <v>24799</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G25" t="s">
@@ -995,21 +1172,24 @@
       <c r="H25">
         <v>6</v>
       </c>
-      <c r="I25" s="1">
-        <v>44587.125</v>
-      </c>
-      <c r="J25" s="1">
-        <v>7431.1875</v>
-      </c>
-    </row>
-    <row r="26" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I25" s="2">
+        <v>47019.15</v>
+      </c>
+      <c r="J25" s="2">
+        <v>7836.5250000000005</v>
+      </c>
+    </row>
+    <row r="26" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C26">
+        <v>20</v>
+      </c>
       <c r="D26" t="s">
         <v>2</v>
       </c>
       <c r="E26">
         <v>24802</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G26" t="s">
@@ -1018,21 +1198,24 @@
       <c r="H26">
         <v>6</v>
       </c>
-      <c r="I26" s="1">
-        <v>83363.5</v>
-      </c>
-      <c r="J26" s="1">
-        <v>13893.916666666666</v>
-      </c>
-    </row>
-    <row r="27" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I26" s="2">
+        <v>87910.599999999991</v>
+      </c>
+      <c r="J26" s="2">
+        <v>14651.766666666665</v>
+      </c>
+    </row>
+    <row r="27" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C27">
+        <v>21</v>
+      </c>
       <c r="D27" t="s">
         <v>3</v>
       </c>
       <c r="E27">
         <v>24798</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G27" t="s">
@@ -1041,21 +1224,24 @@
       <c r="H27">
         <v>6</v>
       </c>
-      <c r="I27" s="1">
-        <v>109375.75</v>
-      </c>
-      <c r="J27" s="1">
-        <v>18229.291666666668</v>
-      </c>
-    </row>
-    <row r="28" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I27" s="2">
+        <v>115341.7</v>
+      </c>
+      <c r="J27" s="2">
+        <v>19223.616666666665</v>
+      </c>
+    </row>
+    <row r="28" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C28">
+        <v>22</v>
+      </c>
       <c r="D28" t="s">
         <v>4</v>
       </c>
       <c r="E28">
         <v>24995</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F28" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G28" t="s">
@@ -1064,21 +1250,24 @@
       <c r="H28">
         <v>6</v>
       </c>
-      <c r="I28" s="1">
-        <v>134776.125</v>
-      </c>
-      <c r="J28" s="1">
-        <v>22462.6875</v>
-      </c>
-    </row>
-    <row r="29" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I28" s="2">
+        <v>142127.54999999999</v>
+      </c>
+      <c r="J28" s="2">
+        <v>23687.924999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C29">
+        <v>23</v>
+      </c>
       <c r="D29" t="s">
         <v>5</v>
       </c>
       <c r="E29">
         <v>24994</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G29" t="s">
@@ -1087,21 +1276,24 @@
       <c r="H29">
         <v>6</v>
       </c>
-      <c r="I29" s="1">
-        <v>176452.375</v>
-      </c>
-      <c r="J29" s="1">
-        <v>29408.729166666668</v>
-      </c>
-    </row>
-    <row r="30" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I29" s="2">
+        <v>186077.05</v>
+      </c>
+      <c r="J29" s="2">
+        <v>31012.841666666664</v>
+      </c>
+    </row>
+    <row r="30" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C30">
+        <v>24</v>
+      </c>
       <c r="D30" t="s">
         <v>6</v>
       </c>
       <c r="E30">
         <v>24801</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="1" t="s">
         <v>34</v>
       </c>
       <c r="G30" t="s">
@@ -1110,21 +1302,24 @@
       <c r="H30">
         <v>6</v>
       </c>
-      <c r="I30" s="1">
-        <v>274690.625</v>
-      </c>
-      <c r="J30" s="1">
-        <v>45781.770833333336</v>
-      </c>
-    </row>
-    <row r="31" spans="4:10" x14ac:dyDescent="0.25">
+      <c r="I30" s="2">
+        <v>289673.75</v>
+      </c>
+      <c r="J30" s="2">
+        <v>48278.958333333336</v>
+      </c>
+    </row>
+    <row r="31" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C31">
+        <v>25</v>
+      </c>
       <c r="D31" t="s">
         <v>7</v>
       </c>
       <c r="E31">
         <v>24800</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="3" t="s">
         <v>34</v>
       </c>
       <c r="G31" t="s">
@@ -1133,11 +1328,11 @@
       <c r="H31">
         <v>6</v>
       </c>
-      <c r="I31" s="1">
-        <v>407932.25</v>
-      </c>
-      <c r="J31" s="1">
-        <v>67988.708333333328</v>
+      <c r="I31" s="2">
+        <v>430183.1</v>
+      </c>
+      <c r="J31" s="2">
+        <v>71697.183333333334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>